<commit_message>
Bill expected per-leg time and energy instead of pack capacity
Recharge energy was keyed to installed pack capacity (reserve and storm
buffer refilled every leg); storms cost no time anywhere. Both battery
strategies now bill the energy a leg consumes in expectation, and the
tender case carries an expected storm ride-out per leg (new route.storm_frac,
placeholder 0.02): it lengthens the leg, idles the waiting tender, and adds
a pack drain the tender refills. Sizing margins (energy_reserve,
storm_duration_h) are capex/mass only, matching the fuel cases' nominal burn.
All expected-value weather parameters are to be calibrated by a voyage
Monte Carlo over historical weather with SoC tracking (see TODO).
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -1493,7 +1493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1505,16 +1505,17 @@
     <col width="23" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1565,50 +1566,55 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>storm_frac</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>standoff_nm</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>idle_h</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>optimize_param</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>optimize_lo</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>optimize_hi</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>optimize_n</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>sweep_param</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>sweep_lo</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>sweep_hi</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>sweep_n</t>
         </is>
@@ -1649,32 +1655,32 @@
       <c r="H2" t="n">
         <v>18</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>op_v_kn</t>
         </is>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>5</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>22</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>18</v>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>d_km</t>
         </is>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>500</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>18000</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>36</v>
       </c>
     </row>
@@ -1713,32 +1719,32 @@
       <c r="H3" t="n">
         <v>18</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>op_v_kn</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>5</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>22</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>18</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>d_km</t>
         </is>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>500</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>18000</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>36</v>
       </c>
     </row>
@@ -1777,35 +1783,32 @@
       <c r="H4" t="n">
         <v>18</v>
       </c>
-      <c r="I4" t="n">
-        <v>12</v>
-      </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>op_v_kn</t>
         </is>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>5</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>22</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>18</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>d_km</t>
         </is>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>500</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>18000</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>36</v>
       </c>
     </row>
@@ -1844,35 +1847,32 @@
       <c r="H5" t="n">
         <v>18</v>
       </c>
-      <c r="I5" t="n">
-        <v>12</v>
-      </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>op_v_kn</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>5</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>22</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>18</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>d_km</t>
         </is>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>500</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>18000</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>36</v>
       </c>
     </row>
@@ -1908,32 +1908,32 @@
       <c r="G6" t="n">
         <v>0.2</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>op_v_kn</t>
         </is>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>5</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>22</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>18</v>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>d_km</t>
         </is>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>500</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>18000</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>36</v>
       </c>
     </row>
@@ -1969,32 +1969,32 @@
       <c r="G7" t="n">
         <v>0.2</v>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>op_v_kn</t>
         </is>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>5</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>22</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>18</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>d_km</t>
         </is>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>500</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>18000</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2033,32 +2033,32 @@
       <c r="H8" t="n">
         <v>18</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>op_v_kn</t>
         </is>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>5</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>22</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>18</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>d_km</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>500</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>18000</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2101,37 +2101,40 @@
         <v>12</v>
       </c>
       <c r="J9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K9" t="n">
         <v>200</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>12</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>op_v_kn</t>
         </is>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>5</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>22</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>18</v>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>d_km</t>
         </is>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>500</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>18000</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2174,9 +2177,12 @@
         <v>12</v>
       </c>
       <c r="J10" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K10" t="n">
         <v>200</v>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace storm ride-out with a floating-tether detach model
The tether floats unloaded, so weather that drops it is far more common
than weather that stops the ship — and a detached ship sails on from its
pack at speed. Detached hours therefore cost the ship no voyage time
(hove-to survival weather moves into availability, which hits every case
alike); the cost lands entirely on the tender, which loses delivery hours
yet must push the crossing plus the final coastal leg's charge through
the cable in the attached window that remains. Renames storm_duration_h/
storm_frac to detach_duration_h/detach_frac: the pack's detach buffer is
sized to the longest continuous cable-dropped stretch, free whenever the
coastal sub-leg already needs a bigger pack.
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -1504,8 +1504,8 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
@@ -1561,12 +1561,12 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>storm_duration_h</t>
+          <t>detach_duration_h</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>storm_frac</t>
+          <t>detach_frac</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">

</xml_diff>